<commit_message>
Update debates data - 2026-06-01
</commit_message>
<xml_diff>
--- a/Debats_Jura.xlsx
+++ b/Debats_Jura.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -41,209 +41,85 @@
     <t xml:space="preserve">Text</t>
   </si>
   <si>
-    <t xml:space="preserve">373559</t>
+    <t xml:space="preserve">374432</t>
   </si>
   <si>
     <t xml:space="preserve">N</t>
   </si>
   <si>
-    <t xml:space="preserve">Page Pierre-André</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FR</t>
+    <t xml:space="preserve">Ryser Franziska</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SG</t>
   </si>
   <si>
     <t xml:space="preserve">DE</t>
   </si>
   <si>
-    <t xml:space="preserve">Le président (Page Pierre-André, président): La session spéciale est ouverte. Nous accueillons aujourd'hui six nouveaux membres de notre conseil. J'ai le plaisir de saluer Mme Michèle Dünki-Bättig, Mme Laura Gantenbein, Mme Miriam Locher, Mme Anna-Béatrice Schmaltz, M. Arbër Bullakaj et M. Loïc Dobler. Je donne la parole à M. Golay pour le bureau.
+    <t xml:space="preserve">Mindestlöhne wurden nicht aus einer Laune heraus eingeführt, sie sind eine Antwort auf reale Probleme im Arbeitsmarkt, auf die Tatsache, dass Menschen Vollzeit arbeiten und trotzdem zu wenig Geld zum Leben verdienen. Mit dieser Vorlage wollen Sie dieses Instrument unterlaufen. Zumindest der Ständerat hat eingesehen, dass die Übersteuerung demokratisch legitimierter Entscheidungen höchst kritisch ist. Die Ausnahme für Mindestlöhne, die bereits vor dieser Gesetzesvorlage beschlossen wurden, wie et</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mindestlöhne wurden nicht aus einer Laune heraus eingeführt, sie sind eine Antwort auf reale Probleme im Arbeitsmarkt, auf die Tatsache, dass Menschen Vollzeit arbeiten und trotzdem zu wenig Geld zum Leben verdienen. Mit dieser Vorlage wollen Sie dieses Instrument unterlaufen. Zumindest der Ständerat hat eingesehen, dass die Übersteuerung demokratisch legitimierter Entscheidungen höchst kritisch ist. Die Ausnahme für Mindestlöhne, die bereits vor dieser Gesetzesvorlage beschlossen wurden, wie etwa in den Kantonen Genf, Neuenburg, Basel-Stadt oder Jura, ist ein Kompromiss für die Vergangenheit und ein kleiner Schritt in Richtung einer demokratisch verträglichen Vorlage. Dieser Schritt muss nun aber konsequent weitergedacht werden. 
+Mit der Minderheit Amoos wird auch für die Zukunft ein solcher Kompromiss gefunden. Wird ein Mindestlohn beschlossen, so erhalten die Sozialpartner Zeit, um zu reagieren. Sie können bei der nächsten Verhandlung der GAV die Löhne anpassen. Spätestens aber nach zwei Jahren müssen die Löhne auf das Niveau der geltenden Mindestlöhne angehoben werden. Das schafft Verbindlichkeit, und es schafft Fairness. Denn ohne klare Fristen besteht die Gefahr, dass über Jahre hinweg zu tiefe Löhne bestehen bleiben. Und genau das ist aus unserer Sicht nicht akzeptabel. Mindestlöhne sind keine symbolischen Grössen, sie sind eine verbindliche Untergrenze. Sie sollen sicherstellen, dass Arbeit vor Armut schützt. Und so kommen wir auch wieder näher zurück an die Verfassung. Denn die Kantone haben gemäss Bundesverfassung das Recht, Mindestlöhne einzuführen. Eine Übersteuerung durch privatrechtliche Verträge - ein allgemeinverbindlich erklärter GAV ist nichts anderes - ist schlicht nicht verfassungskonform. Mit der Minderheit Amoos könnte man die Vorlage schon beinahe als demokratisch verträglich bezeichnen. Deshalb unterstützen wir den Antrag der Minderheit bei Artikel 1 Absatz 4 für einen Lohnschutz, der seinen Namen auch verdient.
 </t>
   </si>
   <si>
-    <t xml:space="preserve">373560</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Golay Roger</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M. Loïc Dobler est le premier suppléant de la liste 1 Parti socialiste jurassien (PSJ). M. Dobler est chef de service à l'Établissement cantonal des assurances sociales du canton du Jura (ECAS Jura). Le gouvernement de la République et canton du Jura l'a proclamé élu par arrêté du 24 mars 2026. Le bureau a constaté que l'élection de M. Loïc Dobler, né le 7 avril 1987, originaire de Mümliswil-Ramiswil dans le canton de Soleure, domicilié à Glovelier, a été validée. M. Dobler remplace notre ancien</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M. Loïc Dobler est le premier suppléant de la liste 1 Parti socialiste jurassien (PSJ). M. Dobler est chef de service à l'Établissement cantonal des assurances sociales du canton du Jura (ECAS Jura). Le gouvernement de la République et canton du Jura l'a proclamé élu par arrêté du 24 mars 2026. Le bureau a constaté que l'élection de M. Loïc Dobler, né le 7 avril 1987, originaire de Mümliswil-Ramiswil dans le canton de Soleure, domicilié à Glovelier, a été validée. M. Dobler remplace notre ancien collègue Pierre-Alain Fridez. Sur la base des indications communiquées par M. Dobler, le bureau n'a identifié aucune activité incompatible avec l'exercice d'un mandat parlementaire au sens de l'article 144 de la Constitution fédérale et de l'article 14 de la loi sur le Parlement. Il propose dès lors de constater formellement l'élection de M. Loïc Dobler.
+    <t xml:space="preserve">374445</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dobler Loïc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le canton du Jura a introduit un salaire minimum cantonal auquel les conventions collectives de travail de force obligatoire peuvent déroger. Vous avez évoqué dans votre intervention, Monsieur le conseiller national, le fait de vouloir redynamiser le partenariat social. Je peux vous dire que la réalité cantonale fait qu'il y a eu zéro convention collective de travail de plus et qu'on a dû introduire des contrats-types de travail dans le secteur de la vente ainsi que d'autres, actuellement en con</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le canton du Jura a introduit un salaire minimum cantonal auquel les conventions collectives de travail de force obligatoire peuvent déroger. Vous avez évoqué dans votre intervention, Monsieur le conseiller national, le fait de vouloir redynamiser le partenariat social. Je peux vous dire que la réalité cantonale fait qu'il y a eu zéro convention collective de travail de plus et qu'on a dû introduire des contrats-types de travail dans le secteur de la vente ainsi que d'autres, actuellement en consultation, dans celui de l'horlogerie. Pouvez-vous donc nous expliquer la notion visant à redynamiser le partenariat social en faisant fi des décisions populaires prises dans les cantons ?
 </t>
   </si>
   <si>
-    <t xml:space="preserve">373693</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Michaud Gigon Sophie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G</t>
+    <t xml:space="preserve">374452</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feller Olivier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RL</t>
   </si>
   <si>
     <t xml:space="preserve">VD</t>
   </si>
   <si>
-    <t xml:space="preserve">Par cette initiative, le canton du Jura demande que la législation fédérale soit adaptée pour interdire les importations de denrées alimentaires dont les méthodes de production ne respecteraient pas les normes en vigueur en Suisse. On y retrouve l'esprit de l'initiative populaire "Fair-Food" : exiger la même chose des importations que de l'agriculture suisse, plus d'équité et de durabilité. "Fair-Food" voulait mettre de la justice dans nos assiettes. Un bénéfice qui vise les producteurs et l'env</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Par cette initiative, le canton du Jura demande que la législation fédérale soit adaptée pour interdire les importations de denrées alimentaires dont les méthodes de production ne respecteraient pas les normes en vigueur en Suisse. On y retrouve l'esprit de l'initiative populaire "Fair-Food" : exiger la même chose des importations que de l'agriculture suisse, plus d'équité et de durabilité. "Fair-Food" voulait mettre de la justice dans nos assiettes. Un bénéfice qui vise les producteurs et l'environnement à l'étranger, comme les familles de l'agriculture, ici en Suisse. La Suisse romande avait soutenu cette initiative en 2018, alors qu'elle était rejetée au niveau suisse.
-Depuis plusieurs années, un élément prépondérant de la politique étrangère suisse a été la multiplication des accords de libre-échange avec d'autres pays. Prenons par exemple les accords avec l'Indonésie et le Mercosur, pour les plus récents. Il s'agit d'acteurs dont les standards agricoles, que ce soit en matière de protection de l'environnement ou de bien-être animal, ne sont en aucun cas équivalents à ceux en vigueur dans notre pays, malgré certaines provisions prévues dans les accords. Cela a des conséquences non négligeables pour l'agriculture suisse. Moins compétitive, notamment en raison des coûts de production plus élevés, elle est soumise à une concurrence qui peut être déloyale vis-à-vis des produits étrangers lorsque ceux-ci ne respectent pas les mêmes normes. L'initiative du canton du Jura s'est inscrite dans le contexte de la révolte paysanne face à ces revenus et ces conditions de marché, et a été déposée en mars 2024, l'idée centrale étant l'équité économique et la défense de l'agriculture suisse.
-Face à cette situation, il faut reconnaître que les solutions déjà en place ont montré leurs limites. Ainsi, les labels et étiquetages d'aliments stigmatisant certaines pratiques sont moins complets que des règles plus contraignantes s'appliquant à tous les acteurs sur le marché suisse. Si les standards agricoles suisses sont stricts, notamment pour freiner les impacts environnementaux, les standards appliqués par certains pays peuvent causer de véritables dommages, détruisant la biodiversité ou soumettant les travailleuses et les travailleurs à des conditions de travail inacceptables. En autorisant ces importations, la Suisse cautionne ces méthodes. Refuser les denrées agricoles qui ne répondent pas à certains standards, c'est, à notre échelle, prendre nos responsabilités pour une agriculture plus écologique et humaine au niveau mondial. C'est aussi renforcer la protection des agriculteurs et des agricultrices suisses face à une concurrence déloyale.
-Pour ces deux raisons, l'impact à l'étranger comme la concurrence pour l'agriculture suisse, une minorité de votre Commission de l'économie et des redevances vous enjoint à donner suite à cette initiative du canton du Jura.
+    <t xml:space="preserve">Il existe des conventions collectives de travail dans le domaine du nettoyage. Il me semble que ces conventions, sauf erreur, sont plutôt négociées sur le plan régional ou cantonal.
+Prenons l'exemple d'une convention connue sur le plan national, celle qui concerne l'hôtellerie-restauration. Comment voulez-vous que le partenariat social puisse continuer de vivre pleinement et de jouer pleinement son rôle si, après de dures négociations entre associations d'employeurs et syndicats, et après avoir </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il existe des conventions collectives de travail dans le domaine du nettoyage. Il me semble que ces conventions, sauf erreur, sont plutôt négociées sur le plan régional ou cantonal.
+Prenons l'exemple d'une convention connue sur le plan national, celle qui concerne l'hôtellerie-restauration. Comment voulez-vous que le partenariat social puisse continuer de vivre pleinement et de jouer pleinement son rôle si, après de dures négociations entre associations d'employeurs et syndicats, et après avoir demandé au Conseil fédéral de rendre la convention collective obligatoire pour toute la branche de l'hôtellerie-restauration, on introduit un salaire minimum qui contourne l'un des éléments de la convention collective de travail ?
+La convention de l'hôtellerie et de la restauration concerne aussi le canton du Jura. Selon la majorité de la commission, en acceptant notre projet vous revivifiez le partenariat social, y compris dans le canton du Jura, puisque, dans ce canton, la convention nationale pour l'hôtellerie-restauration est également appliquée.
 </t>
   </si>
   <si>
-    <t xml:space="preserve">373698</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pamini Paolo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mi esprimo a nome della Commissione dell'economia e dei tributi sull'oggetto 24.326, l'iniziativa cantonale del Canton Giura "Una politica federale 'a deforestazione zero'".
-Die Initiative fordert den Bund auf, das Bundesrecht so anzupassen, dass Rohstoffe und ihre Nebenprodukte, die auf dem Schweizer Markt in Verkehr gebracht werden oder für den Export bestimmt sind, nicht mit Entwaldung in Verbindung stehen.
-Konkret geht es darum, die EU-Verordnung für entwaldungsfreie Produkte (EU Regulation </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mi esprimo a nome della Commissione dell'economia e dei tributi sull'oggetto 24.326, l'iniziativa cantonale del Canton Giura "Una politica federale 'a deforestazione zero'".
-Die Initiative fordert den Bund auf, das Bundesrecht so anzupassen, dass Rohstoffe und ihre Nebenprodukte, die auf dem Schweizer Markt in Verkehr gebracht werden oder für den Export bestimmt sind, nicht mit Entwaldung in Verbindung stehen.
-Konkret geht es darum, die EU-Verordnung für entwaldungsfreie Produkte (EU Regulation on Deforestation-free Products - EUDR), ins Schweizer Recht zu übernehmen. Diese verbietet die Vermarktung von Produkten, die mit Entwaldung in Zusammenhang stehen, wie etwa Palmöl, Kakao, Kaffee, Rindfleisch, Kautschuk und Holz. Die Begründung des Kantons Jura ist zweifach. Einerseits sollen Wettbewerbsnachteile für Schweizer Unternehmen vermieden werden, die in die EU exportieren. Andererseits soll ein Beitrag zur globalen Bekämpfung der Entwaldung sowie zum Schutz der Biodiversität geleistet werden.
-La commission, par 16 voix contre 7 et 2 abstentions, vous propose de ne pas donner suite à l'initiative. Les principales motivations sont les suivantes. L'initiative entraînerait une incertitude réglementaire. Vu que l'application du règlement européen a déjà été reportée à plusieurs reprises, procéder dès à présent à une reprise anticipée entraînerait une incertitude quant à sa mise en oeuvre. Il y aurait aussi des problèmes au niveau des charges administratives élevées. La traçabilité de la certification "sans déforestation" impliquerait des coûts significatifs pour les entreprises, en particulier pour les PME. Finalement, l'initiative aurait une portée très large. Il ne s'agirait pas uniquement des produits suisses, mais également des matières premières, importées et transformées dans notre pays, avec des effets systématiques sur des secteurs économiques entiers.
-Une minorité de la commission vous propose en revanche de donner suite à l'initiative. Je pense que ma collègue, Mme la conseillère nationale Sophie Michaud Gigon, va vous en expliquer les motivations.
-Permettetemi tuttavia una considerazione importante che è stata sollevata anche durante i lavori commissionali. 
-Il mondo sta diventando sempre più verde. Ci sono dati satellitari della Nasa, in particolare le serie storiche Modis e precedenti, che mostrano a partire dagli anni Ottanta un continuo inverdimento della terra e un continuo aumento della massa forestale. La letteratura scientifica di alto livello è chiara su questo punto. Non abbiamo un problema di deforestazione e di diminuzione della vegetazione a livello globale. Lo studio intitolato "Greening of the earth and its drivers" pubblicato su "Nature Climate Change" nel 2016 da Zhu e altri coautori, evidenzia che nel periodo dal 1982 al 2009 tra il 25 per cento e il 50 per cento delle superfici vegetate del pianeta mostra un aumento della copertura fogliare, mentre solo una minima parte registra un declino. Lo stesso studio attribuisce circa il 70 per cento di questo inverdimento all'aumento della concentrazione di anidride carbonica, che agisce come fertilizzante, aumentando la fotosintesi. Forse non tutti ne sono coscienti, ma l'anidride carbonica è il miglior fertilizzante delle piante perché è quello che le piante mangiano. 
-Ulteriori studi su riviste come "Nature Sustainability", "Nature Reviews Earth and Environment", nonché "Nature Climate Change" confermano con dati dal 1981 fino al 2020 e paper pubblicati pochi anni fa, che il fenomeno è reale. I fattori principali sono l'aumento di anidride carbonica, la gestione del territorio e i cambiamenti climatici. In altre parole, la CO2 non è solo un fattore climatico, ma è un input fondamentale per la crescita vegetale, perché è il cibo delle piante. La CO2, alla prova dei fatti, è uno dei migliori fertilizzanti. Questo non vuol dire negare il problema della deforestazione, ma va messo in una chiara prospettiva.
-Vor diesem Hintergrund beantragt Ihnen die Kommission, der Initiative keine Folge zu geben. Sie erachtet eine einseitige Übernahme der europäischen Regelung zum jetzigen Zeitpunkt als verfrüht und mit erheblichen Belastungen verbunden.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">373704</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cette initiative vise à adapter la législation en vigueur pour garantir que les matières premières et produits mis sur le marché suisse ne soient pas issus de la déforestation. Elle vise à lutter contre la déforestation importée. Certains produits, comme le cacao, le soja, le café, la viande bovine ou l'huile de palme, peuvent occasionner à large échelle une déforestation de forêts tropicales. Celles-ci sont pourtant essentielles pour les populations et pays concernés, mais aussi pour l'humanité</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cette initiative vise à adapter la législation en vigueur pour garantir que les matières premières et produits mis sur le marché suisse ne soient pas issus de la déforestation. Elle vise à lutter contre la déforestation importée. Certains produits, comme le cacao, le soja, le café, la viande bovine ou l'huile de palme, peuvent occasionner à large échelle une déforestation de forêts tropicales. Celles-ci sont pourtant essentielles pour les populations et pays concernés, mais aussi pour l'humanité comme puits de carbone. Cette initiative du canton du Jura a trait non seulement à la responsabilité des entreprises, mais aussi à la mise en conformité des entreprises suisses aux normes du marché européen.
-Elle s'inscrit en particulier dans le contexte de la mise en oeuvre prochaine du règlement européen sur la déforestation adopté par les instances de l'Union européenne en 2023. Ce règlement prévoit de nouvelles mesures de diligence pour les opérateurs du marché européen utilisant des matières premières telles que cacao, caoutchouc ou bois. Ces nouvelles obligations toucheront principalement les grandes entreprises et consisteront à prouver systématiquement, notamment par la communication de leurs origines géographiques, que les matières premières utilisées ne sont pas issues de la déforestation. Ces dispositions, qui vont plus loin que celles prévues actuellement par le droit suisse, s'appliqueront aussi aux acteurs d'États tiers qui souhaitent exporter vers l'Union européenne. Se pose donc la question fondamentale de la continuité de l'accès au marché européen pour les entreprises suisses. Le Conseil fédéral se repose sur l'absence actuelle de reconnaissance mutuelle pour éviter de devoir adapter les règles en vigueur. Pourtant, l'expérience nous a montré qu'une position attentiste contient des risques non négligeables.
-Nous nous souvenons de la situation de certains secteurs économiques, comme le secteur biomédical, lors de l'arrêt des négociations sur l'accord-cadre avec l'Union européenne. L'absence de reconnaissance mutuelle dans le domaine médical et celui des biotechnologies a fait capoter de nombreux projets et mis en péril des entreprises suisses pourtant florissantes jusqu'alors. La minorité de la Commission de l'économie et des redevances veut éviter qu'une telle situation ne se répète. En entamant dès maintenant le processus législatif en ce sens, nous pourrons disposer d'une base solide lorsque le moment sera venu de négocier une reconnaissance mutuelle avec l'Union européenne. Même de grandes entreprises suisses, qui seraient pourtant les plus touchées par une telle réglementation, s'y sont déclarées favorables. La proactivité est donc de mise pour obtenir à terme une reconnaissance mutuelle et la garantie de l'accès au marché européen.
-Enfin, donner suite à cette initiative ne permettrait pas seulement de faciliter l'accès des entreprises au marché européen, mais aussi de renforcer significativement la protection de l'environnement. La gestion et la diminution de l'impact environnemental de la Suisse en dehors de ses frontières restent aujourd'hui encore le parent pauvre de notre politique environnementale. Reprendre à notre compte les dispositifs mis en place par l'Union européenne nous permettrait de réaliser des progrès significatifs dans ce domaine sans contraintes disproportionnées. Je le rappelle, les forêts primaires représentent une richesse en biodiversité inestimable ainsi que des puits de carbone plus efficaces. Une politique suisse "Zéro déforestation" est donc un pas vers une prise de responsabilité environnementale allant de la production de matières premières à la consommation finale. C'est un engagement de notre pays en faveur du climat et de la biodiversité.
-Ainsi, je vous enjoins, au nom de la minorité de la Commission de l'économie et des redevances, de donner suite à cette initiative du canton du Jura.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">373714</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hübscher Martin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Die Standesinitiative des Kantons Jura wurde am 14. November 2024 eingereicht. Sie verlangt, den Import von Lebensmitteln, deren Herstellung nicht den Schweizer Vorschriften entspricht, zu verbieten. Die Kommission für Wirtschaft und Abgaben des Nationalrates hat an ihrer Sitzung vom 10. Februar 2026 die vom Kanton Jura eingereichte Standesinitiative vorgeprüft. Der Nationalrat ist Zweitrat. Der Ständerat hat der Standesinitiative am 18. Dezember 2025 auf Antrag seiner Kommission mit 32 zu 10 St</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Die Standesinitiative des Kantons Jura wurde am 14. November 2024 eingereicht. Sie verlangt, den Import von Lebensmitteln, deren Herstellung nicht den Schweizer Vorschriften entspricht, zu verbieten. Die Kommission für Wirtschaft und Abgaben des Nationalrates hat an ihrer Sitzung vom 10. Februar 2026 die vom Kanton Jura eingereichte Standesinitiative vorgeprüft. Der Nationalrat ist Zweitrat. Der Ständerat hat der Standesinitiative am 18. Dezember 2025 auf Antrag seiner Kommission mit 32 zu 10 Stimmen bei 1 Enthaltung keine Folge gegeben. 
-Die Kommissionsmehrheit hält die Forderung der Standesinitiative aus mehreren Gründen für problematisch. Eine Regelung, wonach nur noch nach Schweizer Vorschriften produzierte Lebensmittel importiert werden dürften, stünde nicht nur im Widerspruch zum WTO-Recht, sondern hätte auch eine deutliche Senkung der Versorgung in der Schweiz zur Folge. Verschiedene, auch pflanzliche Produkte wären in der Schweiz kaum in ausreichender Menge verfügbar. Dies würde den Einkaufstourismus verstärken. Zudem wären die Umsetzung und die Kontrolle eines Importverbots sehr schwierig und kaum realisierbar. 
-Auch importierte Lebensmittel müssen dem Schweizer Recht entsprechen; das ist in Artikel 2 des Lebensmittelgesetzes geregelt. Ausgenommen sind jedoch Verfahren und Produktionsmethoden, die sich nicht in den physischen Eigenschaften des Produkts niederschlagen. Deshalb dürfen z. B. Eier aus Batteriehaltung gemäss geltendem Recht importiert werden. Das ist in der Tat ein bisschen störend, aber die Schweiz verfolgt bereits heute eine andere Strategie. Wir setzen auf Deklaration statt auf Verbote. Das hat sich im Grundsatz bewährt. Die Konsumentinnen und Konsumenten haben dadurch die Wahlfreiheit. Neben der Deklaration ist auch die Einführung von Schweizer Nachhaltigkeitsstandards möglich, wie wir das z. B. bei verschiedenen Labels bereits kennen - sei das Bio Suisse, IP-Suisse oder der Branchenstandard Swissmilk Green bei der Milch. Der Weg über die Deklarationspflicht ist richtig. Er ist zwar nicht umfassend, aber er führt indirekt in gewisser Weise auch dazu, dass das Anliegen der Initiative erfüllt werden kann. Das sehen wir beispielsweise beim Kaninchenfleisch oder bei den Eiern.
-Ein komplettes Importverbot von Lebensmitteln, die nicht Schweizer Standards entsprechen, wäre nicht umsetzbar und würde, wie bereits erwähnt, bei etlichen Produkten zu Versorgungslücken führen.
-Eine Kommissionsminderheit will der Standesinitiative Folge geben, um die Bedeutung der Lebensmittelsicherheit und des fairen Wettbewerbs zwischen der Schweizer und der ausländischen Landwirtschaft zu unterstreichen. Beides würde gerade im Zusammenhang mit neuen Handelsabkommen der Schweiz - z. B. mit den USA oder den Mercosur-Staaten - in Zukunft an Aktualität gewinnen.
-Die Kommission beantragt Ihnen mit 15 zu 6 Stimmen bei 3 Enthaltungen, der Standesinitiative keine Folge zu geben. Eine Minderheit beantragt, ihr Folge zu geben. Dieser Antrag wird jetzt gleich durch Frau Michaud Gigon begründet. Herzlichen Dank, wenn Sie der Initiative keine Folge geben.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">373721</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pfister Gerhard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M-E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Es gibt zwei gleichlautende Standesinitiativen aus Basel-Landschaft und Basel-Stadt. Im Kanton Basel-Landschaft ist in der Verfassung verankert, dass sich alle politischen Behörden dafür einzusetzen haben, dass der Kanton Basel-Landschaft zwei Standesstimmen erhalten soll.
-Im Ständerat wurde die Standesinitiative am 16. Juni 2025 ohne Gegenantrag abgelehnt, nachdem die SPK-S einstimmig den Antrag gestellt hatte, ihr keine Folge zu geben. Die SPK Ihres Rates hat die Initiative am 23. Oktober 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Es gibt zwei gleichlautende Standesinitiativen aus Basel-Landschaft und Basel-Stadt. Im Kanton Basel-Landschaft ist in der Verfassung verankert, dass sich alle politischen Behörden dafür einzusetzen haben, dass der Kanton Basel-Landschaft zwei Standesstimmen erhalten soll.
-Im Ständerat wurde die Standesinitiative am 16. Juni 2025 ohne Gegenantrag abgelehnt, nachdem die SPK-S einstimmig den Antrag gestellt hatte, ihr keine Folge zu geben. Die SPK Ihres Rates hat die Initiative am 23. Oktober 2025 beraten. Sie hat Kenntnis von der Debatte im Ständerat wie auch von der Diskussion in der SPK-S genommen, in der eine Vertretung des Kantons Basel-Stadt angehört worden war.
-Der Aufbau des Schweizer Staats und die föderalistische Struktur sind das Resultat von Entscheiden in einer geschichtlichen Epoche und der Entwicklung innerhalb der Geschichte. Insofern ist es selbstverständlich absolut legitim, diese historisch gewachsene Ordnung immer wieder darauf hin zu prüfen, ob sie weiter wachsen und anders gestaltet werden soll. Schliesslich hat der neu geschaffene Kanton Jura selbstverständlich zwei Standesstimmen erhalten. Damals wurde den Halbkantonen auf ihr Begehren hin, ebenfalls eine volle Standesstimme zu erhalten, seitens des Bundesrates beschieden, die Totalrevision der Bundesverfassung abzuwarten. Diese Revision schaffte dann zwar den Status der Halbkantone ab, änderte aber nichts daran, dass den historischen Halbkantonen im Ständerat nur je ein Sitz zugestanden wird.
-Insofern ist der Wunsch aus den Kantonen mit einer Standesstimme eine Art Perpetuum mobile der Vergeblichkeit. Beschränkt sich der Wunsch, wie bei dieser Initiative, auf gewisse Kantone wie Basel-Landschaft und Basel-Stadt, wird er mehrheitlich mit dem Argument abgelehnt, wenn schon müsste er für alle Kantone mit einer Standesstimme gelten. Die Minderheitssprecherin aus dem Kanton Basel-Landschaft hat denn auch ein Kommissionspostulat mit diesem Inhalt beantragt. Dieser Antrag wurde mit 15 zu 7 Stimmen bei 1 Enthaltung abgelehnt. Gibt es aber diese Forderung, wird sie abgelehnt, da ihre Annahme faktisch eine Stärkung der eher konservativen, ländlich geprägten Kantone und eine Stärkung der Deutschschweiz gegenüber der Romandie zur Folge hätte, was wiederum das Gleichgewicht in der Schweizer Eidgenossenschaft stören würde.
-Diese beiden Argumente waren dann auch in der SPK Ihres Rates und im Ständerat die zentralen, warum auch diese Standesinitiative abgelehnt wurde. Unabhängig davon, ob man zwei Standesstimmen für eine begrenzte Anzahl von Kantonen oder für alle will, die Mehrheit im Ständerat sowie in der SPK des Nationalrates erachtet es jetzt als nicht opportun, an dieser historisch gewachsenen Ordnung etwas zu ändern - auch in der vermutlich sehr realistischen Erwartung, dass eine solche Änderung keine Mehrheit im Volk, ganz sicher aber nicht bei den Ständen finden würde. Wer das anders sieht, kann mit einer Volksinitiative versuchen, die Probe aufs Exempel zu machen. Das alles ist nicht zynisch gemeint, sondern einfach realpolitisch. Vermutlich sehen alle hier, die von der Bevölkerung aus den Kantonen Basel-Stadt oder Basel-Landschaft gewählt sind, die Sache anders - mit der vollen politischen Legitimität.
-Die Staatspolitische Kommission Ihres Rates beantragt Ihnen mit 18 zu 4 Stimmen bei 1 Enthaltung, der Initiative keine Folge zu geben.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">373725</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marti Samira</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bitte entschuldigen Sie meine Stimmlage. Ich bin etwas erkältet; darum habe ich mir auch erlaubt, einen Becher für den Notfall mitzunehmen. 
-Die vorliegende Standesinitiative des Kantons Basel-Stadt verlangt, wie der Kommissionssprecher ausgeführt hat, dass die beiden Basel zu Kantonen mit vollem Ständerecht aufgewertet werden. Im Namen der Minderheit und auch im Namen der beiden Kantone bitte ich Sie, diese Standesinitiative zu unterstützen und damit dem Grundsatz zuzustimmen, dass das Thema de</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bitte entschuldigen Sie meine Stimmlage. Ich bin etwas erkältet; darum habe ich mir auch erlaubt, einen Becher für den Notfall mitzunehmen. 
-Die vorliegende Standesinitiative des Kantons Basel-Stadt verlangt, wie der Kommissionssprecher ausgeführt hat, dass die beiden Basel zu Kantonen mit vollem Ständerecht aufgewertet werden. Im Namen der Minderheit und auch im Namen der beiden Kantone bitte ich Sie, diese Standesinitiative zu unterstützen und damit dem Grundsatz zuzustimmen, dass das Thema der Kantone mit halber Standesstimme endlich ernsthaft aufs staatspolitische Tapet gehört. 
-Das Thema beschäftigt unsere Region seit Jahrzehnten. Aufschwung bekam die Debatte aber vor allem auch wieder mit der Gründung des Kantons Jura 1979. Die Eidgenossenschaft entschied damals, nicht zwei Halbkantone, den Kanton Bern und den Kanton Jura, zu gründen und die Standesstimmen zwischen den beiden aufzuteilen, sondern den beiden Kantonen die Gleichbehandlung zu gewähren und zwei Standesstimmen zuzugestehen. Damit wurde damals auch die Zusammensetzung des Ständerates verändert. Anders war es damals bei der Gründung meines Kantons, des Kantons Basel-Landschaft. Die Ländler wehrten sich damals - eine kleine Geschichtsstunde für Sie - erfolgreich gegen die Besetzung durch die Städter. 1832 wurde per Volksabstimmung der Kanton Basel-Landschaft gegründet und dann 1833 nach einem für die Städter verlustreichen Gefecht mit einem entsprechenden Beschluss der Tagsatzung endgültig auch durchgesetzt. Die beiden ehemaligen Halbkantone erhielten dann je eine Stimme im Ständerat. Knapp 150 Jahre später wurde mit der Gründung des Kantons Jura gewissermassen das offizielle Bekenntnis zum Ende der Geschichte der Halbkantone gesetzt. Schon damals monierten die Vertretungen aus dem Kanton Basel-Landschaft, wie es sich denn nun mit ihrem Kanton verhalte, wann sie jetzt endlich gleichbehandelt würden. Der damals zuständige Bundesrat Furgler vertröstete sie, die Frage könne man dann im Rahmen der nächsten Totalrevision der Bundesverfassung diskutieren. Er wolle, sagte er verständlicherweise, jetzt die Gründung des Kantons Jura nicht gefährden. Dann wurden die Halbkantone im Rahmen der Totalrevision zwar abgeschafft und die Gleichheit der Kantone und das Gebot der Gleichbehandlung der Kantone festgehalten, aber das Relikt der sogenannt vollwertigen Kantone mit halber Standesstimme blieb bestehen. 2001 wurde der parlamentarischen Initiative Janiak 01.403, "Basel-Landschaft und Basel-Stadt. Vollberechtigte Kantone", vom Nationalrat ebenfalls keine Folge gegeben. Auch damals wurde dagegen vor allem eingewendet, dass die Verfassung des Kantons Basel-Stadt damals noch das Ziel der Wiedervereinigung beinhaltete. Basel-Land strebte bereits damals die zwei Sitze an, Basel-Stadt aber den Zusammenschluss. Mehr als zehn Jahre später wurde über eine Initiative zur Wiedervereinigung abgestimmt. Basel-Stadt nahm diese an, Basel-Land aber lehnte sie mit über 70 Prozent ab. Unterdessen wurde auch die Verfassung des Kantons Basel-Stadt angepasst. Die Wiedervereinigung ist nun kein offizielles Verfassungsziel mehr, nur die gute Zusammenarbeit. All das zeigt, dass sich seit der Debatte in den 70er-Jahren die Situation auch vor Ort geändert hat und sich beide Kantone als vollwertige und auch selbstständige Kantone verstehen. In der Region wird nicht verstanden, warum man im Unterschied zu praktisch allen anderen Kantonen nur einen Sitz im Ständerat hat und man quasi vom Nachbarkanton Jura, der uns nahe ist und den wir gut kennen, links überholt wurde. 
-Mir ist klar, dass diese Standesinitiative Schwächen hat. Sie klärt nicht, warum neue Ungleichheiten mit den anderen Kantonen mit halber Standesstimme, den Appenzeller Kantonen sowie Nid- und Obwalden, geschaffen werden sollen. Auch das Argument der wirtschaftlichen Stärke, das in der Begründung der Initiative vom Kanton Basel-Stadt genannt wird, überzeugt mich persönlich nicht. Die Standesvertretung soll bekanntlich ja nicht an Wirtschaftsleistung oder an Grösse geknüpft werden. Ich bedauere deshalb - der Kommissionssprecher hat das ebenfalls erwähnt -, dass die Kommission meinen Antrag auf ein Postulat nicht unterstützt hat. Es braucht eine ernsthafte Auslegeordnung zu Reformoptionen, wie die Gleichbehandlung der Regionen bzw. der Kantone unter Berücksichtigung des Gleichgewichts im Bundesstaat erreicht werden können. Das ist keine statische Angelegenheit, die über hundert Jahre genau das gleiche Gleichgewicht darstellt. Sie werden mit mir einverstanden sein, dass die Konfession heute zum Beispiel nicht mehr die entscheidende Konfliktlinie in unserem Bundesstaat ist. Es sind andere Unterschiedlichkeiten, die wir überwinden und über die wir als Bundesstaat zusammenhalten müssen. Es sind sprachliche und kulturelle Differenzen, die es in einem vielfältigen Land wie der Schweiz gibt. Lassen Sie uns darüber nachdenken. Diese Standesinitiative könnte dafür der Anfang sein. 
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">374283</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rosenwasser Anna</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Die Demokratie-Initiative verlangt, dass Ausländerinnen und Ausländer nach fünf Jahren in der Schweiz das Recht auf Einbürgerung erhalten. Die Bedingung ist, dass sie nach diesen fünf Jahren eine Landessprache beherrschen, die Sicherheit nicht gefährden und nicht ins Gefängnis müssen. 
-Momentan kann ein Viertel aller Menschen, die in der Schweiz leben, weder abstimmen noch wählen, geschweige denn für ein politisches Amt kandidieren. Das heisst, über 2 Millionen Menschen in der Schweiz sind zwar </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Die Demokratie-Initiative verlangt, dass Ausländerinnen und Ausländer nach fünf Jahren in der Schweiz das Recht auf Einbürgerung erhalten. Die Bedingung ist, dass sie nach diesen fünf Jahren eine Landessprache beherrschen, die Sicherheit nicht gefährden und nicht ins Gefängnis müssen. 
-Momentan kann ein Viertel aller Menschen, die in der Schweiz leben, weder abstimmen noch wählen, geschweige denn für ein politisches Amt kandidieren. Das heisst, über 2 Millionen Menschen in der Schweiz sind zwar von politischen Entscheiden betroffen, dürfen aber nicht mitbestimmen. Wer hier zuhause ist, ist von hier. Diese Aussage ist nicht radikal, denn es geht nicht um unsere Wurzeln. Diejenigen, über die bestimmt wird, müssen mitbestimmen können. Wenn drei Viertel unseres Landes über das andere Viertel bestimmen, ist das keine vollwertige Demokratie. 
-Das aktuell geltende Einbürgerungsrecht ist eine Lotterie. Je nach Kanton hat man ein bisschen Glück oder sehr viel Pech. Im Aargau und im Kanton St. Gallen kostet es über 2000 Franken, sich einbürgern zu lassen, im Kanton Zug nur 350 Franken. Im Kanton Jura wurde eine Person von einer Einbürgerungskommission abgelehnt, weil sie am Sonntag Rasen gemäht hat. In Zürich wurde jemand nicht angenommen, weil er den geografischen und historischen Ursprung von Raclette nicht kannte. In Arth, in Schwyz, wurde jemand abgelehnt, weil er nicht wusste, dass Wölfe und Bären sich im Tierpark Goldau ein Gehege teilen. Es braucht endlich einheitliche Regeln gegen diese Willkür. Es sagt nichts über uns aus, ob wir wissen, welche Tiere sich ein Gehege teilen, aber es sagt viel über uns aus, mit wem wir ein Land teilen. 
-Wer einen Schweizer Pass hat, kann nicht nur wählen und abstimmen, es geht um Grundrechte. Eine Staatsbürgerschaft gibt einem Menschen Sicherheit - Sicherheit, hier bleiben zu dürfen, eine Familie zu gründen, die Meinung zu äussern, sich frei zu bewegen. Ein Viertel unserer Bevölkerung kann das momentan nicht. Wenn sie einen Schweizer Pass wollen, wird es teuer, dauert ewig und ist voller Willkür und Schikane. 
-Seien wir ehrlich, der einzige Grund, weswegen wir das tolerieren, ist, dass viele dieser Ausländerinnen und Ausländer nicht weiss genug oder nicht reich genug sind. Wenn es um Ausländer geht, wird gern bis nach links argumentiert, dass diese ja schliesslich auch Steuern zahlen und hier arbeiten würden und dass wir ohne sie verloren wären, etwa auf dem Bau, im Gastgewerbe oder in der Pflege. Und das stimmt: Ohne migrantische Menschen wären wir alle aufgeschmissen. Aber das ist nicht der Grund, warum Menschen ohne Schweizer Pass einen einheitlichen Anspruch auf Einbürgerung erhalten sollen. Ausländerinnen und Ausländer müssen uns nichts nützen. 
-Ich bin für die Demokratie-Initiative, weil ich meinen Mitmenschen auf Augenhöhe begegnen will, nicht, weil ich von ihnen profitiere. Wer mit mir im gleichen Land lebt, soll mitbestimmen können, egal, ob er in Herrliberg oder in Spreitenbach wohnt, egal, ob er Thomas oder Mahmoud heisst, und egal, ob er meiner Meinung ist oder irgendeinen Gugus abstimmt. Ich respektiere nämlich nicht nur Menschen, die ähnlich sind wie ich, sondern alle. 
-Zuletzt noch dies: Wenn Ausländerinnen und Ausländer fünf Jahre lang friedlich sein müssen, um sich den Pass zu verdienen, wie es die Initiative verlangt, könnten wir Schweizerinnen und Schweizer unseren Pass eigentlich abgeben, wenn wir uns innerhalb von fünf Jahren mal menschenverachtend verhalten. Aber dann wäre unsere Demokratie wieder unvollständiger - und dieser Saal um einiges leerer. 
-Ich bitte Sie, die Demokratie-Initiative anzunehmen.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">374382</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tuosto Brenda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Suisse romande refuse de payer le prix d'une planification défaillante des CFF et de l'Office fédéral des transports (OFT) pendant une décennie. L'horaire 2025 n'est pas une simple mise à jour technique, c'est un choix politique. Un choix politique de priorisation entre les différentes régions, entre les différentes vitesses, entre transport de voyageurs et transport de marchandises. Il est inadmissible qu'une partie du pays soit contrainte de porter seule le poids de choix politiques de refo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Suisse romande refuse de payer le prix d'une planification défaillante des CFF et de l'Office fédéral des transports (OFT) pendant une décennie. L'horaire 2025 n'est pas une simple mise à jour technique, c'est un choix politique. Un choix politique de priorisation entre les différentes régions, entre les différentes vitesses, entre transport de voyageurs et transport de marchandises. Il est inadmissible qu'une partie du pays soit contrainte de porter seule le poids de choix politiques de refonte de l'horaire. Si les CFF invoquent des problèmes de ponctualité pour justifier ces mesures, ces désagréments ne se justifient absolument pas et ne sauraient être absorbés au seul profit du poumon économique alémanique indûment épargné. En interrompant la liaison IC5 entre Genève et Olten, l'OFT impose aux habitantes et habitants du nord de la Suisse jusqu'à l'ouest du pays une accessibilité au rail dégradée pour la décennie à venir. On ne peut exiger de la Suisse occidentale qu'elle sacrifie sa connectivité pour compenser des retards d'infrastructures qui ne lui incombent pas. L'introduction de l'horaire 2025 marque une régression pour les habitantes et habitants de la ligne du Pied-du-Jura. L'allongement des trajets d'environ 8 pour cent sur toutes les lignes romandes d'importance nationale et la fin des liaisons directes contredisent les objectifs de neutralité carbone de l'Office fédéral de l'environnement. La complexification des parcours est un frein majeur à l'attractivité du rail.
-Le Département fédéral de l'environnement, des transports, de l'énergie et de la communication (DETEC) tente de nous rassurer en parlant de la mise en service du tunnel de Gléresse et de la remise en place du train circulant via le by-pass comme d'une révolution de l'horaire 2030. Restons lucides face à ces éléments de communication qui masquent la réalité du terrain. Le projet de by-pass existait déjà dans Rail 2000. Présenter un simple retour à la normale après travaux comme une avancée stratégique est une lecture un peu trop sélective de la réalité. D'autant plus que l'horaire 2030 ne prévoit aucun rétablissement des correspondances entre la ligne du Pied-du-Jura et celle du Valais, laissant la rupture de charge inchangée à Lausanne. La situation reste donc problématique pour les déplacements de l'Arc jurassien au-delà de Martigny. L'axe du Pied-du-Jura doit être connecté avec des noeuds de correspondance à Zurich, à Bâle et à Lausanne. Les régions d'Argovie, de Soleure, du Jura bernois, du Jura, des deux Bâle, de Neuchâtel et du Nord vaudois doivent rester connectées avec le reste de la Suisse.
-Avec ce postulat, je demande formellement le rétablissement des correspondances entre l'IC5 et l'IR90. Un réseau national n'a de sens que si ses noeuds fonctionnent. Il faut corriger cette erreur de planification maintenant. Le Conseil fédéral nous promet des solutions pour 2030, mais elles sont insuffisantes. Aujourd'hui, l'inertie administrative du DETEC bloque les projets déjà approuvés comme ceux liés à la redondance Lausanne-Genève, à la halte d'Y-Parc ou aux mesures de compensation des 100 millions de francs qui ont été votées ces dernières années et qui pourraient améliorer rapidement la situation. Si nous attendons une nouvelle décision des chambres en 2027 voire 2028, ces études deviendront caduques. Nous allons gaspiller l'argent public en refaisant de nouvelles études déjà payées. Je demande au Conseil fédéral de débloquer ces mesures immédiatement pour sauver ce qui peut l'être.
-En conclusion, nous ne demandons pas de faveur. Nous demandons le respect des engagements pris envers la Suisse occidentale et la Suisse alémanique. L'horaire 2025 est une situation qui, sans intervention politique, deviendra la norme : des liaisons nationales interrompues et des durées de trajet rallongées. Il ne s'agit pas d'exiger des offres ou des investissements supplémentaires, mais simplement de revenir à la normale. La situation d'avant 2025 doit être remise en place totalement et maintenant. Soutenir ce postulat, c'est répondre à l'appel de l'Alliance des villes et des milieux économiques situés sur l'ensemble de l'axe du Pied-du-Jura. La cohésion nationale ne saurait se maintenir si l'on consent à l'isolement d'une grande partie du pays. Je vous remercie pour votre soutien.
+    <t xml:space="preserve">374592</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crevoisier Crelier Mathilde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La présente motion part d'un constat aussi simple que dramatique : à la retraite, l'écart de revenu moyen entre femmes et hommes double d'un seul coup pour passer de 16 pour cent d'inégalité salariale à 31 pour cent d'écart de rente. Ainsi, les femmes retraitées perçoivent en moyenne un tiers de moins que les hommes, soit 36 108 francs contre 52 488 francs, selon les chiffres de 2023. Cet écart important est entièrement imputable à la prévoyance professionnelle, car la différence entre femmes et</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La présente motion part d'un constat aussi simple que dramatique : à la retraite, l'écart de revenu moyen entre femmes et hommes double d'un seul coup pour passer de 16 pour cent d'inégalité salariale à 31 pour cent d'écart de rente. Ainsi, les femmes retraitées perçoivent en moyenne un tiers de moins que les hommes, soit 36 108 francs contre 52 488 francs, selon les chiffres de 2023. Cet écart important est entièrement imputable à la prévoyance professionnelle, car la différence entre femmes et hommes dans l'AVS est quasiment nulle. Cet écart ne diminue pas depuis plusieurs années. En comparaison internationale, la Suisse pointe à un peu reluisant cinquième rang des pays européens présentant les plus fortes différences de retraite entre les femmes et les hommes.
+Afin de combler ce fossé, la présente motion visait donc à tenir compte des lacunes de rente découlant des tâches éducatives et d'assistance, qui sont assumées majoritairement par les femmes au détriment de leur épargne-vieillesse, et d'introduire dans la loi sur la prévoyance professionnelle vieillesse, survivants et invalidité (LPP) le principe de la bonification ; principe bien connu et reconnu puisqu'il existe déjà dans l'AVS, comme l'a rapporté le rapporteur de commission. Comme cela a été dit, cette motion s'inscrivait dans la série d'interventions déposées dans le sillage du refus de la révision de la LPP en 2024 ; interventions qui avaient toutes été renvoyées à la commission compétente et qui ont été retirées, que ce soit en commission ou aujourd'hui au conseil, au profit du postulat 26.3521 de la CSSS, que nous avons accepté tout à l'heure.
+Ainsi, au vu des considérations avancées dans le postulat de la commission, qui refuse une approche isolée au profit d'une réflexion globale sur les améliorations possibles dans la LPP, et au vu des arguments du Conseil fédéral, qui oeuvre d'ores et déjà à la nouvelle révision de la LPP et cherche lui aussi des solutions pour améliorer la prévoyance professionnelle des personnes travaillant un temps partiel ou ayant de faibles revenus, parmi lesquels les femmes sont justement surreprésentées, je me rallie au mouvement initié par les autres auteurs de motion et retire la présente motion, dans l'espoir toutefois que les mesures de la prochaine réforme permettent enfin d'infléchir cet écart important, qui n'a plus lieu d'être dans le système de rente moderne d'un pays prospère comme le nôtre.
 </t>
   </si>
 </sst>
@@ -298,8 +174,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I11" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I5" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I5"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -631,7 +507,7 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46139</v>
+        <v>46174</v>
       </c>
       <c r="C2" t="s">
         <v>10</v>
@@ -652,268 +528,94 @@
         <v>15</v>
       </c>
       <c r="I2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46139</v>
+        <v>46174</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G3" t="s">
         <v>14</v>
       </c>
       <c r="H3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46140</v>
+        <v>46174</v>
       </c>
       <c r="C4" t="s">
         <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
         <v>14</v>
       </c>
       <c r="H4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="I4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46140</v>
+        <v>46174</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E5" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F5" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="G5" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="H5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
         <v>32</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>46140</v>
-      </c>
-      <c r="C6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" t="s">
-        <v>33</v>
-      </c>
-      <c r="I6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>46140</v>
-      </c>
-      <c r="C7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H7" t="s">
-        <v>38</v>
-      </c>
-      <c r="I7" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>46140</v>
-      </c>
-      <c r="C8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" t="s">
-        <v>41</v>
-      </c>
-      <c r="E8" t="s">
-        <v>42</v>
-      </c>
-      <c r="F8" t="s">
-        <v>43</v>
-      </c>
-      <c r="G8" t="s">
-        <v>14</v>
-      </c>
-      <c r="H8" t="s">
-        <v>44</v>
-      </c>
-      <c r="I8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>46</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>46140</v>
-      </c>
-      <c r="C9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" t="s">
-        <v>47</v>
-      </c>
-      <c r="E9" t="s">
-        <v>48</v>
-      </c>
-      <c r="F9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H9" t="s">
-        <v>50</v>
-      </c>
-      <c r="I9" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>52</v>
-      </c>
-      <c r="B10" s="1" t="n">
-        <v>46142</v>
-      </c>
-      <c r="C10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" t="s">
-        <v>53</v>
-      </c>
-      <c r="E10" t="s">
-        <v>48</v>
-      </c>
-      <c r="F10" t="s">
-        <v>37</v>
-      </c>
-      <c r="G10" t="s">
-        <v>14</v>
-      </c>
-      <c r="H10" t="s">
-        <v>54</v>
-      </c>
-      <c r="I10" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>56</v>
-      </c>
-      <c r="B11" s="1" t="n">
-        <v>46142</v>
-      </c>
-      <c r="C11" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" t="s">
-        <v>57</v>
-      </c>
-      <c r="E11" t="s">
-        <v>48</v>
-      </c>
-      <c r="F11" t="s">
-        <v>24</v>
-      </c>
-      <c r="G11" t="s">
-        <v>14</v>
-      </c>
-      <c r="H11" t="s">
-        <v>58</v>
-      </c>
-      <c r="I11" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update debates data - 2026-06-04
</commit_message>
<xml_diff>
--- a/Debats_Jura.xlsx
+++ b/Debats_Jura.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -292,6 +292,21 @@
 Je ne suis pas non plus un fan absolu de ce projet. J'aurais peut-être dû d'emblée dire que je suis président de l'intergroupe parlementaire Feu bleu, qui regroupe en particulier les sapeurs-pompiers, qui attendent ce genre de données actualisées au jour le jour. Actuellement, quand il y a des travaux dans les villes ou dans les grandes villes, ils doivent envoyer un de leurs membres régulièrement circuler dans leur secteur d'activité pour savoir si les chemins habituels sont disponibles ou non en fonction des travaux qu'il y a. Aujourd'hui, ce n'est pas acceptable. Ce projet mérite donc quand même un peu plus que d'être simplement abandonné sans avoir été approfondi.
 Je le répète, pour moi, il y a deux éléments qui sont absolument fondamentaux. En ce qui concerne la fourniture des informations, soit tous les acteurs doivent fournir leurs informations, soit ce n'est pas le cas. Si on laisse la possibilité de le faire ou pas, si on n'oblige pas à fournir les données, ce projet n'a pas de sens. C'est pour moi un élément assez essentiel. En ce qui concerne les moyens dont on parle pour le mettre en oeuvre, les 28 EPT et les coûts qui sont prévus sont absolument exorbitants. On n'a pas arrêté de nous dire, y compris de la part de l'administration, que l'intelligence artificielle allait nous permettre de gagner, mais qu'on ne sait pas exactement combien. Ce sont des questions qui, à mon avis, méritent d'être encore discutées en commission avant de couler ce projet. Je serai le premier à reconnaître, si on n'a pas de réponses claires et concrètes notamment sur ces deux éléments-là, lors du vote final, qu'il ne faut pas soutenir ce projet, si on n'a pas pu l'améliorer dans ces deux domaines. Cependant, aujourd'hui, je ne suis pas en mesure de vous dire ni de vous recommander s'il faut soutenir ou non ce projet parce qu'à mon avis, la commission n'est pas allée assez loin dans le travail d'examen. J'avais par exemple proposé que l'on fasse des auditions des milieux concernés. C'est vrai que si on ne veut pas entrer en matière, ce n'est pas la peine qu'on perde notre temps à faire des auditions, mais je pense que si nous avions été un peu plus loin et notamment avions procédé à ces auditions, peut-être que nous aurions un autre regard sur ce projet qui, je le répète, mérite d'être amélioré et que, sans ces améliorations, je ne soutiendrai pas non plus lors du vote final.
 Aujourd'hui, je vous invite vraiment à entrer en matière.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">375342</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permettez-moi d'apporter quelques mots en français dans ce débat qui semble surtout concerné les Suisses alémaniques, alors qu'il concerne toute la Suisse, tous les cantons suisses et tous les citoyens de ce pays. Oui, personne ne conteste que le 8 mars dernier, une majorité du peuple a accepté la réforme qui lui était proposée au travers de l'imposition individuelle. Oui, le peuple a voulu mettre un terme à cette inégalité qui durait depuis bien trop longtemps. Cependant, le peuple était mis de</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permettez-moi d'apporter quelques mots en français dans ce débat qui semble surtout concerné les Suisses alémaniques, alors qu'il concerne toute la Suisse, tous les cantons suisses et tous les citoyens de ce pays. Oui, personne ne conteste que le 8 mars dernier, une majorité du peuple a accepté la réforme qui lui était proposée au travers de l'imposition individuelle. Oui, le peuple a voulu mettre un terme à cette inégalité qui durait depuis bien trop longtemps. Cependant, le peuple était mis devant un choix cornélien ; vraiment cornélien. Beaucoup de gens, lors de la campagne, ont choisi cette option de peur de voir cette inégalité se poursuivre.
+Ce choix cornélien, vous le connaissez : il était d'accepter de mettre un terme à cette inégalité et d'accepter un modèle compliqué qui crée d'autres inégalités et qui conduit à des divisions, souvent antisociales, ou de refuser cette réforme et voir cette inégalité encore se poursuivre. On peut d'ailleurs se poser la question : pourquoi le texte de l'initiative dont on parle aujourd'hui n'a-t-il pas été traité simultanément à l'initiative sur l'imposition individuelle ? En effet, dans ce cas, le peuple aurait eu un vrai choix sur le modèle qu'il entend. Se contentait-il de régler une inégalité sur le plan fédéral qui dure depuis trop longtemps, ou bien voulait-il révolutionner le système fiscal, ce dont je ne suis absolument pas certain pour avoir discuté avec les gens ?
+Le peuple a tranché pour cette solution. Toutefois, aujourd'hui, soutenir l'initiative qui vous est proposée ne remet pas en cause la fin de cette inégalité entre les couples mariés et les autres, au contraire, et n'a pas d'incidence sur l'organisation familiale, contrairement à ce qu'on a pu entendre. Elle offre au peuple un véritable choix sur le modèle : régler un problème fédéral sans créer de nouvelles inégalités ou mettre en place un système bureaucratique sans amélioration claire pour une grande majorité des contribuables. Si l'initiative de rang constitutionnel est acceptée, elle rendra caduque la révision législative acceptée par le peuple. C'est assez clair pour ceux qui en douteraient ou qui auraient émis des avis contraires aujourd'hui.
+Il nous appartiendra à nous, parlementaires, de trouver une solution plus simple, plus égalitaire, comme les cantons l'ont fait, sans leur imposer, au passage, une révolution dont une majorité d'entre eux n'a pas voulu. Accepter l'initiative, ce n'est pas trahir la volonté du peuple, mais, au contraire, c'est lui donner l'occasion de choisir la méthode.
+Quant aux coûts, pour essayer de répondre à Madame Herzog, vous savez très bien que cela dépendra du modèle qui sera retenu par le Parlement. Ce coût, dans le débat sur l'imposition individuelle, a aussi évolué. Il pourra aussi évoluer dans les débats que nous aurons. Pour l'instant, la question se pose sur la méthode : comment régler cette inégalité qui dure depuis aussi longtemps ?
+Dans ce cadre-là, je vous invite à soutenir la proposition de la minorité, qui offrira un vrai choix au Parlement et à la population sur la méthode et sur le coût.
 </t>
   </si>
 </sst>
@@ -346,8 +361,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I15" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I16" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I16"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1076,6 +1091,35 @@
         <v>72</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="1" t="n">
+        <v>46177</v>
+      </c>
+      <c r="C16" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" t="s">
+        <v>64</v>
+      </c>
+      <c r="E16" t="s">
+        <v>39</v>
+      </c>
+      <c r="F16" t="s">
+        <v>20</v>
+      </c>
+      <c r="G16" t="s">
+        <v>20</v>
+      </c>
+      <c r="H16" t="s">
+        <v>74</v>
+      </c>
+      <c r="I16" t="s">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-06-10
</commit_message>
<xml_diff>
--- a/Debats_Jura.xlsx
+++ b/Debats_Jura.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -195,12 +195,12 @@
   </si>
   <si>
     <t xml:space="preserve">Le postulat Bally vise à réformer la valorisation fiscale des immeubles par les cantons en Suisse et, en réalité, à l'uniformiser sur le plan fédéral. Cette proposition avait plus de sens probablement avant la votation du 28 septembre 2025 sur la valeur locative, mais, maintenant que la valeur locative a été ou va être supprimée sur décision populaire, naturellement, la question de la valeur fiscale perd de son importance. Toutefois, elle ne perd pas complètement de son importance, puisqu'il reste quand même une valorisation fiscale, notamment au moment de taxer la fortune des citoyens.
-En Suisse, il y a une souveraineté cantonale, notamment en matière fiscale et les cantons restent libres d'imposer la méthode de calcul de la valorisation des immeubles qu'ils souhaitent. Il y a une certaine logique derrière cette approche. D'abord, on n'estime pas de la même manière un immeuble si l'on se trouve dans une région de montagne ou dans une région de plaine, en ville ou à la campagne. Finalement, il y a des choix politiques derrière ces méthodes d'évaluation. Si un franc vaut un franc partout dans le pays, un appartement n'est pas partout estimé de la même manière, son utilisation pouvant varier fortement. Puis, les cantons qui renoncent à une valorisation très haute des immeubles renoncent aussi à l'impôt qui va avec, et c'est un choix cantonal.
-En réalité le postulat qui vous est proposé ne vise naturellement pas à réduire la valorisation fiscale des immeubles ; ne vous y méprenez pas. Le postulat qui vous est proposé vise naturellement à uniformiser vers le haut la valeur des immeubles. C'est une hausse d'impôts que l'on vous propose ici ; une hausse de l'impôt sur la fortune pour tous les propriétaires de ce pays qui aboutit immanquablement à une augmentation des impôts et aussi à une diminution de l'attractivité du statut de propriétaire, que l'on devrait au contraire encourager.
-Pour toutes les familles de notre pays qui sont propriétaires, et il y en a un certain nombre, ces modifications peuvent avoir des impacts très forts sur leur fiche d'impôt, mais sur leur possibilité d'accéder notamment aux subsides des primes maladies. Il n'y a aucun besoin de faire cette réforme aujourd'hui, les cantons sont souverains et s'organisent très bien entre eux.
+En Suisse, il y a une souveraineté cantonale, notamment en matière fiscale, et les cantons restent libres d'imposer la méthode de calcul de la valorisation des immeubles qu'ils souhaitent. Il y a une certaine logique derrière cette approche. D'abord, on n'estime pas de la même manière un immeuble si l'on se trouve dans une région de montagne ou dans une région de plaine, en ville ou à la campagne. Finalement, il y a des choix politiques derrière ces méthodes d'évaluation. Si un franc vaut un franc partout dans le pays, un appartement n'est pas partout estimé de la même manière, son utilisation pouvant varier fortement. Puis, les cantons qui renoncent à une valorisation très haute des immeubles renoncent aussi à l'impôt qui va avec, et c'est un choix cantonal.
+En réalité, le postulat qui vous est proposé ne vise naturellement pas à réduire la valorisation fiscale des immeubles[NB]; ne vous y méprenez pas. Le postulat qui vous est proposé vise naturellement à uniformiser vers le haut la valeur des immeubles. C'est une hausse d'impôts que l'on vous propose ici[NB]; une hausse de l'impôt sur la fortune pour tous les propriétaires de ce pays, qui aboutit immanquablement à une augmentation des impôts et aussi à une diminution de l'attractivité du statut de propriétaire, que l'on devrait au contraire encourager.
+Pour toutes les familles de notre pays qui sont propriétaires, et il y en a un certain nombre, ces modifications peuvent avoir des impacts très forts sur leur fiche d'impôt, mais aussi sur leur possibilité d'accéder notamment aux subsides des primes maladies. Il n'y a aucun besoin de faire cette réforme aujourd'hui, les cantons sont souverains et s'organisent très bien entre eux.
 On vous dit qu'il ne s'agit que d'un postulat, mais ne vous y méprenez pas. Un postulat n'est jamais anodin. Nous allons, en acceptant ce postulat, confier à l'administration le soin d'analyser la situation. Il y aura un rapport et des propositions législatives. Lors de la prochaine réforme de la RPT qui, immanquablement, reviendra, l'administration proposera forcément d'uniformiser les valeurs locatives et la valorisation des immeubles entre les cantons.
-Je vous le dis franchement : nous nous battons contre toute forme de hausse d'impôts, nous ne voulons pas de nouveaux impôts. Même si vous les trouvez justes, Madame Bally, nous préférons des impôts bas injustes à des impôts élevés justes et, dans ces circonstances, nous préférons rejeter un postulat qui introduirait de nouveaux impôts qui vous paraissent justes plutôt que de modifier la loi dans ce sens. Aussi, j'aurais compris si la gauche avait proposé cette réforme, mais venant d'un parti, le Centre, fort dans des cantons qui ont des valorisations raisonnables, proposer cette réforme, c'est en réalité mettre un grain dans la machine qui fonctionne bien aujourd'hui.
-Pour cette raison, je vous invite et je m'adresse en particulier aux élus du Centre, à rejeter cette proposition qui aboutira, qu'on le veuille ou non, à une augmentation des impôts des citoyens.
+Je vous le dis franchement[NB]: nous nous battons contre toute forme de hausse d'impôts, nous ne voulons pas de nouveaux impôts. Même si vous les trouvez justes, Madame Bally, nous préférons des impôts bas injustes à des impôts élevés justes et, dans ces circonstances, nous préférons rejeter un postulat qui introduirait de nouveaux impôts qui vous paraissent justes plutôt que de modifier la loi dans ce sens. Aussi, j'aurais compris si la gauche avait proposé cette réforme, mais, venant d'un parti, le Centre, fort dans des cantons qui ont des valorisations raisonnables, proposer cette réforme, c'est en réalité mettre un grain dans la machine qui fonctionne bien aujourd'hui.
+Pour cette raison, je vous invite, et je m'adresse en particulier aux élus du Centre, à rejeter cette proposition qui aboutira, qu'on le veuille ou non, à une augmentation des impôts des citoyens.
 </t>
   </si>
   <si>
@@ -235,21 +235,21 @@
   </si>
   <si>
     <t xml:space="preserve">La Commission des finances recommande l'adoption des comptes 2025. Le groupe socialiste s'y associe sans réserve. Nous tenons en préambule à remercier l'Administration fédérale des finances pour la qualité de ses travaux et son précieux soutien dans l'accomplissement de notre travail.
-Les comptes sont bons. Le frein à l'endettement est respecté, et même largement respecté. Le frein à l'endettement autorisait un déficit de 262 millions de francs. Le compte ordinaire boucle sur un excédent de 1,185 milliard de francs. Les recettes ont progressé de 4,3 pour cent, les dépenses de 2 pour cent seulement. La Confédération finance la totalité de ses investissements par ses propres moyens sans recourir à l'endettement. La dette nette recule à 16,1 pour cent du PIB et le compte de résultat dépasse largement ce qui était prévu au budget. Ce sont des chiffres solides. Ils méritent d'être posés clairement parce qu'ils contrastent singulièrement avec le tableau qui nous était brossé lors des débats budgétaires récents. Il y a, en effet, quelque chose de troublant dans la séquence que ce Parlement rejoue session après session. À l'automne, la situation financière est décrite comme tendue, contrainte, au bord du déséquilibre, voire pire. Des coupes sont décidées dans les politiques sociales, dans les services publics. Ces choix sont présentés non pas comme des choix, mais comme des nécessités, comme si la comptabilité avait décidé à la place de la politique. Et puis viennent les comptes, et les comptes racontent une autre histoire. On répondra légitimement que le résultat de cette année doit une partie de son éclat à des recettes extraordinaires non reconductibles. C'est exact et ce n'est pas contesté. Mais ce qui n'a rien d'extraordinaire, ce qui, au contraire, est d'une banalité répétitive et prévisible, c'est le schéma lui-même, les prophéties pessimistes de l'automne, les sacrifices qu'elles commandent et les comptes, quelques mois plus tard, qui en révèlent l'exagération. Lorsque l'erreur va systématiquement dans le même sens, elle cesse d'être une erreur, elle devient une méthode. Une méthode qui n'est pas sans conséquences. Derrière chaque décision budgétaire, il y a des réalités concrètes : des familles qui voient leurs prestations diminuer, des cantons qui compensent ce que la Confédération ne finance plus, des régions périphériques dont la cohésion repose sur des services publics que l'on réduit année après année. La méthode voulue par la majorité de notre conseil a un prix, et ce sont toujours les mêmes qui le payent. 
-Le groupe socialiste approuve ces comptes et il sera présent cet automne lorsque s'ouvrira le débat sur le budget 2027, lorsqu'immanquablement les mêmes voix expliqueront que la situation est tendue, que les marges sont inexistantes, qu'il n'y a pas d'autres issues que de couper encore dans les mêmes politiques, sur le dos des mêmes personnes. Ce Parlement a le droit d'assumer ses choix, mais qu'il les assume pour ce qu'ils sont, des choix politiques portés par une majorité, avec des conséquences assumées, et non pas des fatalités déguisées en équations budgétaires. Sous prétexte du "mieux d'État", c'est surtout le "moins d'État" qui est souhaité. En politique, il y a toujours le choix ; la question est de savoir qui le supporte. 
+Les comptes sont bons. Le frein à l'endettement est respecté, et même largement respecté. Le frein à l'endettement autorisait un déficit de 262 millions de francs. Le compte ordinaire boucle sur un excédent de 1,185 milliard de francs. Les recettes ont progressé de 4,3 pour cent, les dépenses de 2 pour cent seulement. La Confédération finance la totalité de ses investissements par ses propres moyens sans recourir à l'endettement. La dette nette recule à 16,1 pour cent du PIB et le compte de résultat dépasse largement ce qui était prévu au budget. Ce sont des chiffres solides. Ils méritent d'être posés clairement, parce qu'ils contrastent singulièrement avec le tableau qui nous était brossé lors des débats budgétaires récents. Il y a, en effet, quelque chose de troublant dans la séquence que ce Parlement rejoue session après session. À l'automne, la situation financière est décrite comme tendue, contrainte, au bord du déséquilibre, voire pire. Des coupes sont décidées dans les politiques sociales, dans les services publics. Ces choix sont présentés non pas comme des choix, mais comme des nécessités, comme si la comptabilité avait décidé à la place de la politique. Et puis viennent les comptes, et les comptes racontent une autre histoire. On répondra légitimement que le résultat de cette année doit une partie de son éclat à des recettes extraordinaires non reconductibles. C'est exact et ce n'est pas contesté. Mais ce qui n'a rien d'extraordinaire, ce qui, au contraire, est d'une banalité répétitive et prévisible, c'est le schéma lui-même[NB]: les prophéties pessimistes de l'automne, les sacrifices qu'elles commandent et les comptes, quelques mois plus tard, qui en révèlent l'exagération. Lorsque l'erreur va systématiquement dans le même sens, elle cesse d'être une erreur, elle devient une méthode, une méthode qui n'est pas sans conséquences. Derrière chaque décision budgétaire, il y a des réalités concrètes[NB]: des familles qui voient leurs prestations diminuer, des cantons qui compensent ce que la Confédération ne finance plus, des régions périphériques dont la cohésion repose sur des services publics que l'on réduit année après année. La méthode voulue par la majorité de notre conseil a un prix, et ce sont toujours les mêmes qui le payent. 
+Le groupe socialiste approuve ces comptes et il sera présent cet automne lorsque s'ouvrira le débat sur le budget 2027, lorsqu'immanquablement les mêmes voix expliqueront que la situation est tendue, que les marges sont inexistantes, qu'il n'y a pas d'autre issue que de couper encore dans les mêmes politiques, sur le dos des mêmes personnes. Ce Parlement a le droit d'assumer ses choix, mais qu'il les assume pour ce qu'ils sont, des choix politiques portés par une majorité, avec des conséquences assumées, et non pas des fatalités déguisées en équations budgétaires. Sous prétexte du "mieux d'État", c'est surtout le "moins d'État" qui est souhaité. En politique, il y a toujours le choix[NB]; la question est de savoir qui le supporte. 
 </t>
   </si>
   <si>
     <t xml:space="preserve">374817</t>
   </si>
   <si>
-    <t xml:space="preserve">Commençons par un constat sans appel : la violence sexiste et sexuelle est un fléau qui n'épargne pas notre pays, comme l'a encore rappelé hier le Conseil fédéral en lançant la deuxième phase de sa campagne contre la violence domestique. En 2025, la police a enregistré 22 000 infractions dues à la violence domestique, un chiffre dont on sait qu'il ne constitue que la partie émergée de l'iceberg et cache une sombre réalité dans laquelle un nombre encore plus élevé de cas n'entrera jamais dans les</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Commençons par un constat sans appel : la violence sexiste et sexuelle est un fléau qui n'épargne pas notre pays, comme l'a encore rappelé hier le Conseil fédéral en lançant la deuxième phase de sa campagne contre la violence domestique. En 2025, la police a enregistré 22 000 infractions dues à la violence domestique, un chiffre dont on sait qu'il ne constitue que la partie émergée de l'iceberg et cache une sombre réalité dans laquelle un nombre encore plus élevé de cas n'entrera jamais dans les statistiques de la criminalité. En effet, l'accès à la justice des victimes de violence sexiste, sexuelle et de violence domestique est encore semé d'embûches. Parmi celles-ci, la prise en charge des victimes par les autorités de procédure pénale, soit la police, les ministères publics et les tribunaux, est souvent pointée du doigt comme un facteur de renoncement pour les victimes à poursuivre la procédure. En cause, on peut mentionner notamment un manque de sensibilité dans l'accueil, la prise en charge et l'audition des victimes avec un risque important de victimisation secondaire pour ces dernières.
+    <t xml:space="preserve">Commençons par un constat sans appel[NB]: la violence sexiste et sexuelle est un fléau qui n'épargne pas notre pays, comme l'a encore rappelé hier le Conseil fédéral, en lançant la deuxième phase de sa campagne contre la violence domestique. En 2025, la police a enregistré 22 000 infractions dues à la violence domestique, un chiffre dont on sait qu'il ne constitue que la partie émergée de l'iceberg et cache une sombre réalité dans laquelle un nombre encore plus élevé de cas n'entrera jamais dans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commençons par un constat sans appel[NB]: la violence sexiste et sexuelle est un fléau qui n'épargne pas notre pays, comme l'a encore rappelé hier le Conseil fédéral, en lançant la deuxième phase de sa campagne contre la violence domestique. En 2025, la police a enregistré 22 000 infractions dues à la violence domestique, un chiffre dont on sait qu'il ne constitue que la partie émergée de l'iceberg et cache une sombre réalité dans laquelle un nombre encore plus élevé de cas n'entrera jamais dans les statistiques de la criminalité. En effet, l'accès à la justice des victimes de violence sexiste, sexuelle et de violence domestique est encore semé d'embûches. Parmi celles-ci, la prise en charge des victimes par les autorités de procédure pénale, soit la police, les ministères publics et les tribunaux, est souvent pointée du doigt comme un facteur de renoncement pour les victimes à poursuivre la procédure. En cause, on peut mentionner notamment un manque de sensibilité dans l'accueil, la prise en charge et l'audition des victimes, avec un risque important de victimisation secondaire pour ces dernières.
 Ainsi, la motion de la Commission des affaires juridiques du Conseil national, "Modification du code de procédure pénale concernant la formation initiale et continue des autorités pénales", vise donc à améliorer cette formation de manière à améliorer l'accès à la justice pour les victimes. Elle se base sur le rapport du Conseil fédéral de 2025, donnant suite au postulat Fehlmann Rielle 21.4215.
-Vous l'avez entendu, la majorité de la commission rejette la motion au motif de la répartition des compétences. Effectivement, les cantons sont responsables de la formation initiale et continue des autorités de poursuite pénale, mais le prétexte du fédéralisme ne saurait nous prémunir d'examiner si nous remplissons nos propres obligations. Que les cantons soient tenus d'assurer la formation continue et initiale, y compris en vertu de l'article 15 de la Convention d'Istanbul, ne signifie pas encore toutefois que celle-ci soit assurée. Or, aujourd'hui, on constate que la mise en oeuvre est, sinon lacunaire, encore inégale. Le rapport de 2022 d'évaluation du Groupe d'experts sur la lutte contre la violence à l'égard des femmes et la violence domestique (Grevio) déplore que la Suisse n'ait toujours pas de programme de formation standardisé dans le domaine de la violence sexuelle pour la police, et que celle-ci soit facultative pour les services judiciaires. Le Grevio encourage vivement les autorités suisses à prendre des mesures afin de veiller à dispenser une formation initiale et continue systématique et obligatoire aux professionnels en lien avec les victimes et les auteurs de toutes les formes de violence visées par la Convention d'Istanbul. Ainsi, si l'argument de la compétence cantonale doit évidemment être pris en compte, il doit aussi être soigneusement sous-pesé en regard de nos responsabilités à l'échelon fédéral.
-Dans le cadre de la réponse au postulat précité, la Confédération a commandé un avis de droit qui conclut que la Confédération dispose d'une marge de manoeuvre en vertu de l'article 123 de la Constitution qui règle la compétence fédérale en matière de droit pénal et de droit de procédure pénale, lorsqu'il s'agit de garantir l'exécution uniforme du droit fédéral, ainsi que la mise en oeuvre du droit international. Or, ces deux conditions sont remplies. D'une part, aujourd'hui, malgré les efforts d'uniformisation consentis par les cantons, force est de constater que la formation des autorités de poursuite pénale est encore trop fragmentée pour assurer l'égalité de traitement des victimes dans l'ensemble du pays et que si la formation initiale de la police est désormais généralisée, celle des ministères publics reste encore lacunaire. D'ailleurs, bien que le Conseil fédéral propose lui aussi de rejeter la motion, il admet qu'il reste des efforts à accomplir, par exemple dans l'audition des victimes ou encore au niveau de la coopération interdisciplinaire et de la formation initiale et continue des acteurs. D'autre part, une intervention de la Confédération au titre de l'article 123 de la Constitution se justifie également par l'obligation qui nous est faite en vertu de l'article 15 de la Convention d'Istanbul de garantir la formation des professionnels. Dès lors, rejeter la présente motion, comme le propose la majorité de la commission, ne relève pas du simple respect des compétences cantonales, mais bien d'une appréciation politique. Or, il faut admettre que la situation actuelle en matière de prise en charge des victimes ne permet ni de garantir l'exécution uniforme du droit ni de remplir nos obligations internationales. C'est également la conclusion à laquelle est parvenu le Conseil national, par 127 voix contre 63 et 1 abstention, soit l'intégralité des groupes parlementaires à une exception près.
+Vous l'avez entendu, la majorité de la commission rejette la motion au motif de la répartition des compétences. Effectivement, les cantons sont responsables de la formation initiale et continue des autorités de poursuite pénale, mais le prétexte du fédéralisme ne saurait nous prémunir d'examiner si nous remplissons nos propres obligations. Que les cantons soient tenus d'assurer la formation continue et initiale, y compris en vertu de l'article 15 de la Convention d'Istanbul, ne signifie pas encore, toutefois, que celle-ci soit assurée. Or, aujourd'hui, on constate que la mise en oeuvre est, sinon lacunaire, encore inégale. Le rapport de 2022 d'évaluation du Groupe d'experts sur la lutte contre la violence à l'égard des femmes et la violence domestique (Grevio) déplore que la Suisse n'ait toujours pas de programme de formation standardisé dans le domaine de la violence sexuelle pour la police, et que celle-ci soit facultative pour les services judiciaires. Le Grevio encourage vivement les autorités suisses à prendre des mesures afin de veiller à dispenser une formation initiale et continue systématique et obligatoire aux professionnels en lien avec les victimes et les auteurs de toutes les formes de violence visées par la Convention d'Istanbul. Ainsi, si l'argument de la compétence cantonale doit évidemment être pris en compte, il doit aussi être soigneusement sous-pesé en regard de nos responsabilités à l'échelon fédéral.
+Dans le cadre de la réponse au postulat précité, la Confédération a commandé un avis de droit qui conclut qu'elle dispose d'une marge de manoeuvre en vertu de l'article 123 de la Constitution qui règle la compétence fédérale en matière de droit pénal et de droit de procédure pénale, lorsqu'il s'agit de garantir l'exécution uniforme du droit fédéral, ainsi que la mise en oeuvre du droit international. Or, ces deux conditions sont remplies. D'une part, aujourd'hui, malgré les efforts d'uniformisation consentis par les cantons, force est de constater que la formation des autorités de poursuite pénale est encore trop fragmentée pour assurer l'égalité de traitement des victimes dans l'ensemble du pays, et que si la formation initiale de la police est désormais généralisée, celle des ministères publics reste encore lacunaire. D'ailleurs, bien que le Conseil fédéral propose lui aussi de rejeter la motion, il admet qu'il reste des efforts à accomplir, par exemple concernant l'audition des victimes ou encore au niveau de la coopération interdisciplinaire et de la formation initiale et continue des acteurs. D'autre part, une intervention de la Confédération au titre de l'article 123 de la Constitution se justifie également par l'obligation qui nous est faite, en vertu de l'article 15 de la Convention d'Istanbul, de garantir la formation des professionnels. Dès lors, rejeter la présente motion, comme le propose la majorité de la commission, ne relève pas du simple respect des compétences cantonales, mais bien d'une appréciation politique. Or, il faut admettre que la situation actuelle en matière de prise en charge des victimes ne permet ni de garantir l'exécution uniforme du droit ni de remplir nos obligations internationales. C'est également la conclusion à laquelle est parvenu le Conseil national, par 127 voix contre 63 et 1 abstention, soit l'intégralité des groupes parlementaires, à une exception près.
 Il a été dit en commission que nous nous rendrions risibles en adoptant cette motion. Le ridicule ne tue pas, contrairement à la violence sexiste et sexuelle qui fait encore et toujours une victime toutes les deux semaines dans notre pays.
 Dans l'intérêt des victimes, mais aussi des autorités chargées de les accompagner dans la procédure pénale, je vous invite à suivre la minorité de la commission et à adopter la motion.
 </t>
@@ -361,11 +361,11 @@
     <t xml:space="preserve">376044</t>
   </si>
   <si>
-    <t xml:space="preserve">Il m'appartient de vous présenter un bref rapport de l'audition que la Commission de gestion a menée avec Mme la conseillère fédérale Karine Keller-Sutter, cheffe du Département fédéral des finances, lors de l'examen du rapport de gestion 2025 du Conseil fédéral. Je concentrerai mon propos sur les deux thèmes choisis par Mme la conseillère fédérale, à savoir la situation des finances fédérales et la réglementation bancaire.
-Premièrement, s'agissant des évolutions et perspectives du budget fédéra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Il m'appartient de vous présenter un bref rapport de l'audition que la Commission de gestion a menée avec Mme la conseillère fédérale Karine Keller-Sutter, cheffe du Département fédéral des finances, lors de l'examen du rapport de gestion 2025 du Conseil fédéral. Je concentrerai mon propos sur les deux thèmes choisis par Mme la conseillère fédérale, à savoir la situation des finances fédérales et la réglementation bancaire.
+    <t xml:space="preserve">Il m'appartient de vous présenter un bref rapport de l'audition que la Commission de gestion a menée avec Mme la conseillère fédérale Karin Keller-Sutter, cheffe du Département fédéral des finances, lors de l'examen du rapport de gestion 2025 du Conseil fédéral. Je concentrerai mon propos sur les deux thèmes choisis par Mme la conseillère fédérale, à savoir la situation des finances fédérales et la réglementation bancaire.
+Premièrement, s'agissant des évolutions et perspectives du budget fédéral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il m'appartient de vous présenter un bref rapport de l'audition que la Commission de gestion a menée avec Mme la conseillère fédérale Karin Keller-Sutter, cheffe du Département fédéral des finances, lors de l'examen du rapport de gestion 2025 du Conseil fédéral. Je concentrerai mon propos sur les deux thèmes choisis par Mme la conseillère fédérale, à savoir la situation des finances fédérales et la réglementation bancaire.
 Premièrement, s'agissant des évolutions et perspectives du budget fédéral pour les années 2027 à 2029, il faut constater une détérioration initiale en 2027. Le budget de l'année 2027 tablait d'abord sur un équilibre, avant d'afficher un déficit structurel estimé entre 400 et 600 millions de francs. Ce recul découle des coupes parlementaires dans le programme de réexamen des tâches - ou Programme d'allègement budgétaire 2027 - ou de l'extension du programme européen Horizon par exemple. 
 Concernant les nouvelles charges, le budget de 2027 subit une aggravation supplémentaire de 400 millions de francs au niveau des dépenses, causée par des corrections d'estimations pour les assurances sociales et la migration. 
 Concernant la détente finale et la stabilisation, on relève que malgré ces hausses de dépenses, une nette embellie du côté des recettes permet d'anticiper une détente pour le budget de 2027. De plus, un équilibre structurel redevient possible pour 2028 et 2029, et l'année 2029 affiche un besoin de correction réduit à 300 millions de francs. 
@@ -383,6 +383,69 @@
 Concernant la réglementation bancaire liée à la crise de Credit Suisse, les pressions des lobbies et le chantier législatif "too big to fail", le Département fédéral des finances a fait de cette réglementation sa priorité. Des travaux majeurs sont en cours, basés sur les propositions du Conseil fédéral, les motions parlementaires et les conclusions de la Commission d'enquête parlementaire , afin de combler les failles des banques d'importance systémique.
 Concernant le lobbying agressif et les pressions sur le Parlement, les parlementaires ont confié s'être sentis soumis à une pression intense et inconfortable de la part des lobbyistes craignant des sanctions financières, notamment la suppression de subventions pour leur parti s'ils soutenaient la réglementation bancaire. Ceci interpelle beaucoup la Commission de gestion.
 Concernant la tentative de déstabilisation des institutions - autre sujet extrêmement critique pour la Commission de gestion -, au-delà du cas de la presse où UBS a retiré ses publicités au journal "Finanz und Wirtschaft" en raison de sa ligne éditoriale, des manoeuvres ont été entreprises pour diviser le Conseil fédéral, à tel point que le gouvernement a exceptionnellement rendu public le fait que les choix qu'il a faits quant au projet de réglementation bancaire se sont faits à l'unanimité. Le Conseil fédéral est conscient qu'il évolue en terrain miné, mais il veut tenir le cap qu'il s'est fixé. Il transmettra bientôt ses propositions au Parlement, ce dont nous lui savons gré.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">376222</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amoos Emmanuel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dans son ensemble, le groupe socialiste accueille favorablement cette révision de la LDFR, qui renforce plusieurs principes fondamentaux que nous défendons depuis longtemps : la protection des terres agricoles contre la spéculation, la pérennisation de l'exploitation à titre personnel et une meilleure reconnaissance des réalités sociales du monde agricole. Le projet corrige certaines inégalités lors des successions, des ventes d'exploitations ou des séparations, en particulier au détriment des é</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dans son ensemble, le groupe socialiste accueille favorablement cette révision de la LDFR, qui renforce plusieurs principes fondamentaux que nous défendons depuis longtemps : la protection des terres agricoles contre la spéculation, la pérennisation de l'exploitation à titre personnel et une meilleure reconnaissance des réalités sociales du monde agricole. Le projet corrige certaines inégalités lors des successions, des ventes d'exploitations ou des séparations, en particulier au détriment des épouses et des veuves.
+Cette révision répond également à une réalité qu'il ne faut pas ignorer : les femmes restent largement sous-représentées à la tête des exploitations agricoles. En Suisse, seules 7,2 pour cent des exploitations sont dirigées par des femmes, un taux parmi les plus faibles d'Europe. Cette situation n'est pas le fruit du hasard, mais le résultat de mécanismes structurels qui continuent de limiter l'accès des femmes, en particulier des filles d'agriculteurs, aux terres, aux exploitations et au patrimoine agricole. De nombreuses études ont montré que les mécanismes de transmission du patrimoine agricole, combinés à des rôles de genre encore très marqués, conduisent à une forte concentration des terres, des bâtiments et des entreprises agricoles entre les mains d'un nombre restreint d'hommes. Les filles d'agriculteurs sont encore trop souvent écartées de la reprise des exploitations ou contraintes de renoncer à une part importante de leur héritage. Toute avancée qui favorise une plus grande équité dans la transmission des exploitations mérite donc d'être saluée.
+Si nous soutenons le projet, nous estimons toutefois que certains ajustements sont encore nécessaires pour mieux atteindre les objectifs de la loi. Les minorités que nous proposons s'inscrivent dans cet esprit. Il s'agit de renforcer la protection de la propriété foncière agricole, favoriser la transmission des exploitations, tout particulièrement aux femmes, et préserver une agriculture familiale vivante, diversifiée et accessible aux générations futures.
+À l'article 9 alinéa 3, nous proposons d'ajouter que toutes les parts sociales de la société de capitaux doivent être détenues par des personnes physiques domiciliées en Suisse. Cette exigence est proportionnée et cohérente avec les objectifs mêmes de la révision. Si nous acceptons que l'exploitation à titre personnel puisse être exercée sous la forme d'une société de capitaux, nous devons également nous assurer que cette ouverture ne crée pas une voie détournée permettant une prise de contrôle, même partielle ou indirecte, de nos terres agricoles par des intérêts étrangers. Les terres agricoles constituent une ressource stratégique pour notre pays. Dans ce contexte, il est légitime d'exiger que les propriétaires des sociétés bénéficiant de ce régime particulier entretiennent un lien réel et durable avec la Suisse.
+À l'article 60 alinéa 1 lettre j, avec ma minorité, nous proposons de tenir compte de la possibilité de construire des bâtiments manquants, nécessaires à l'exploitation, ou de transformer, rénover ou remplacer ceux qui existent, lorsque l'exploitation permet d'assumer les dépenses correspondantes. La rédaction actuelle ne prend en considération que les bâtiments existants pour déterminer si une entreprise agricole peut être divisée. Cette approche est excessivement rigide et risque de freiner inutilement la transmission et le renouvellement des structures agricoles. Si nous voulons maintenir une agriculture familiale dynamique et une population paysanne forte, nous devons accepter que certaines grandes exploitations puissent être partagées entre plusieurs repreneurs lorsque cela est économiquement viable. Sans mécanisme de ce type, l'évolution se fera inévitablement vers des exploitations toujours plus grandes et toujours moins nombreuses. C'est aussi un aspect déterminant si nous voulons que plus de femmes puissent reprendre des exploitations.
+Je vous demande également de soutenir ma minorité à l'article 60 alinéa 2 lettre a. La législation actuelle prévoit déjà des exceptions à l'interdiction du partage matériel lorsqu'il s'agit d'améliorer les structures d'autres entreprises agricoles. En revanche, elle offre peu de souplesse lorsqu'une entreprise existante, notamment de grande taille, ne trouve pas de repreneur et pourrait pourtant être transmise plus facilement après une division adaptée de ses structures.
+Cette modification contribue à favoriser la transmission des exploitations, tout en maintenant des garde-fous clairs contre les partages injustifiés.
+Ma minorité propose encore d'abroger l'article 66 alinéa 2. L'un des objectifs fondamentaux du droit foncier rural est de lutter contre la hausse excessive des prix des terres agricoles et de maintenir ceux-ci à un niveau compatible avec leur exploitation. Or, aujourd'hui, la loi considère déjà qu'un prix est surfait lorsqu'il dépasse de plus de 5 pour cent les valeurs usuelles de la région. Permettre aux cantons de porter cette marge à 15 pour cent affaiblit considérablement ce garde-fou. Dans le contexte actuel, cette souplesse n'apparaît plus justifiée. Les prix du foncier agricole connaissent à nouveau une tendance à la hausse dans plusieurs régions. Dans le canton du Jura, par exemple, les prix ont progressé durant sept années consécutives jusqu'en 2023. La suppression de cette dérogation cantonale constitue une mesure simple, cohérente et efficace pour limiter les risques de spirale haussière. Elle renforce l'application uniforme de la loi et contribue à préserver l'accès à la terre pour les agricultrices et les agriculteurs qui souhaitent exploiter eux-mêmes leur domaine. Un seuil unique à l'échelle nationale évite également les distorsions entre cantons et garantit une application plus prévisible du droit.
+Le groupe socialiste soutiendra l'entrée en matière et la révision dans son ensemble, tout en vous invitant à suivre les minorités que nous avons déposées, ainsi que les minorités Bertschy et II (Michaud Gigon), afin de renforcer encore la protection du foncier agricole et les perspectives de transmission des exploitations.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">376239</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je me permets de prendre la parole puisque je ne figure pas nommément dans cette minorité, mais que je la soutiens également. Je ne vais pas répéter ce qu'a dit M. Rieder. Simplement, je tiens à rappeler que le principe de ligne aérienne a été retiré du projet à la suite de la consultation. Je me permets de citer le message du Conseil fédéral : "Le principe de la ligne aérienne, contenu initialement, était particulièrement contesté et a été retiré du projet. Son maintien aurait entraîné une augm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je me permets de prendre la parole puisque je ne figure pas nommément dans cette minorité, mais que je la soutiens également. Je ne vais pas répéter ce qu'a dit M. Rieder. Simplement, je tiens à rappeler que le principe de ligne aérienne a été retiré du projet à la suite de la consultation. Je me permets de citer le message du Conseil fédéral : "Le principe de la ligne aérienne, contenu initialement, était particulièrement contesté et a été retiré du projet. Son maintien aurait entraîné une augmentation importante du nombre d'exceptions, ce qui aurait réduit à néant l'effet d'accélération recherché." Introduire cette primauté de la ligne aérienne aura donc probablement pour effet de ralentir les procédures plutôt que de les accélérer.
+Je me permets également de rappeler les risques sécuritaires qui peuvent concerner les lignes aériennes. On parle beaucoup de sécurité en ce moment. On renforce les moyens de l'armée. On parle d'attaques éventuelles. Les lignes électriques sont un point stratégique d'une infrastructure nationale. Si elles ne sont pas enterrées, elles sont évidemment plus vulnérables. C'est également un point que l'on peut prendre en considération dans les réflexions.
+La proposition vise simplement à établir ou à rétablir une forme de neutralité ou du moins à envisager sérieusement l'enterrement des lignes. Évidemment, les considérations environnementales entrent aussi en ligne de compte, mais également celles d'aménagement du territoire. Je rappelle quand même qu'on est sur un territoire petit, que des conflits d'utilisation sont nombreux et qu'une ligne à haute tension prend de la place. Cela touche évidemment les zones à bâtir, mais on peut également imaginer que cela interfère avec des infrastructures routières, par exemple. Dès lors, il peut être d'un intérêt, pour de multiples raisons très diversifiées, de considérer sérieusement l'enterrement des lignes à haute tension. 
+C'est pourquoi je vous invite à revenir sur cette décision du Conseil national en adoptant la minorité Rieder, afin d'offrir de meilleures chances aux lignes souterraines lorsqu'elles sont pertinentes.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">376258</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comme l'a dit le rapporteur, cet article 15bbis est un peu le coeur du projet. C'est un des vecteurs qui permettra de réaliser l'accélération des projets d'extension du réseau électrique. Dans ce sens, il s'agit de le concevoir de manière adéquate et aussi équilibrée. Vous voyez que le projet du Conseil fédéral prévoit que les projets d'assainissement ou de remplacement des lignes à haute tension égale ou supérieure à 220 kilovolts - il s'agit donc du réseau de transport à très haute tension - p</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comme l'a dit le rapporteur, cet article 15bbis est un peu le coeur du projet. C'est un des vecteurs qui permettra de réaliser l'accélération des projets d'extension du réseau électrique. Dans ce sens, il s'agit de le concevoir de manière adéquate et aussi équilibrée. Vous voyez que le projet du Conseil fédéral prévoit que les projets d'assainissement ou de remplacement des lignes à haute tension égale ou supérieure à 220 kilovolts - il s'agit donc du réseau de transport à très haute tension - puissent être réalisés sur le tracé existant ou dans la zone qui le jouxte immédiatement. Il s'agit donc déjà d'une amélioration, d'une accélération, puisqu'il ne serait plus nécessaire de repasser par une procédure pour opérer ces travaux. Maintenant, la commission de notre conseil vous propose à l'alinéa 1 d'élargir cette possibilité jusqu'au réseau de 36 kilovolts. Cela inclut donc le niveau de réseau 3, à savoir le réseau à haute tension. Cette disposition concerne donc, en tout, pour le réseau à très haute tension, environ 6000 kilomètres de lignes, et pour le réseau à haute tension, 16 000 kilomètres de lignes. Ce sont déjà, avec la disposition telle qu'elle est prévue à l'alinéa 1, 22 000 kilomètres de lignes qui sont concernées par cette facilitation.
+À l'alinéa 3, qui fait l'objet de ma minorité, la majorité de la commission a décidé d'élargir encore les possibilités, puisqu'elle propose de ne pas tenir compte des distances légales par rapport aux forêts et aux cours d'eau et donc de prévoir que les projets d'assainissement, d'extension ou de remplacement de lignes puissent être réalisés à des distances réduites par rapport aux forêts et aux cours d'eau. Avec cela, on franchit ce point d'équilibre qui doit être maintenu.
+Je vous rappelle que nous avons une discussion qui est similaire à celle concernant le projet de loi pour l'accélération des procédures que nous avons menée l'année passée et qui a attaqué également le droit de recours - on va y revenir. Il est important de maintenir une forme d'équilibre de manière à protéger les intérêts de l'environnement et aussi à éviter de créer une disposition qui est trop déséquilibrée et qui donnerait lieu ensuite à un référendum. Attaquer des exigences légales qui sont déjà relativement minimales dans le droit en vigueur par rapport aux distances des forêts et des cours d'eau, c'est franchir un pas de trop.
+Je vous propose donc de ne pas le faire et d'en rester à la version du Conseil fédéral à l'alinéa 3.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">376340</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il s'agit là d'une autre croisade - et pas la dernière, malheureusement - de la Commission de l'environnement, de l'aménagement du territoire et de l'énergie, qui vise à limiter le droit de recours des associations.
+Je rappelle que, dans ce projet, nous avons déjà considérablement affaibli le droit de l'environnement à l'article 15bbis alinéas 3 et 4, en particulier pour ce qui est de la protection des marais. Maintenant, nous cherchons également à limiter les voies de droit. Comme l'a dit le ra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il s'agit là d'une autre croisade - et pas la dernière, malheureusement - de la Commission de l'environnement, de l'aménagement du territoire et de l'énergie, qui vise à limiter le droit de recours des associations.
+Je rappelle que, dans ce projet, nous avons déjà considérablement affaibli le droit de l'environnement à l'article 15bbis alinéas 3 et 4, en particulier pour ce qui est de la protection des marais. Maintenant, nous cherchons également à limiter les voies de droit. Comme l'a dit le rapporteur de la commission, cette limitation du droit de recours des organisations dans la loi sur le Tribunal fédéral fait écho à la restriction que nous avons déjà opérée lors du traitement du "Beschleunigungserlass", le projet d'accélération des procédures.
+Cela dit, il faut quand même savoir sur quoi cela porte : on parle ici du réseau de raccordement de ces seize centrales hydroélectriques. Si l'on enlève la possibilité de faire recours, on enlève la possibilité de contester des projets qui peuvent s'étendre tel un ruban sur plusieurs dizaines de kilomètres. Je rappelle quand même qu'on parle de centrales qui sont situées en haute montagne et dont l'infrastructure de raccordement peut s'étaler sur de très grandes surfaces, contrairement aux projets de centrales hydroélectriques à proprement parler qui, elles, sont restreintes à un site circonscrit. Donc on cherche à argumenter de l'harmonisation des procédures, mais c'est en occultant le fait que le site et l'infrastructure de raccordement ne sont pas pareils et ne peuvent pas être traités de la même manière. Effectivement, l'administration et l'Office fédéral de l'énergie saluent cette harmonisation, mais je rappelle que quand on a discuté de ces attaques contre le droit de recours dans la loi sur le Tribunal fédéral, l'administration s'y était opposée dans la mesure où c'est une attaque frontale contre le droit de recours des organisations, qui est un peu la base du droit de l'environnement.
+Je rappelle aussi - s'il faut le rappeler - que lorsque la population avait été invitée à valider ces seize projets de centrales dans la loi sur l'approvisionnement en électricité, la brochure de votation indiquait que le droit de recours des associations était garanti. C'est donc aussi dans ce cadre-là que s'inscrit cette nouvelle restriction du droit de recours.
+Enfin, j'aimerais rappeler qu'avec les décisions que nous avons prises aujourd'hui, nous restreignons déjà le droit de recours dans la loi sur les installations électriques. Il s'agit d'une part de l'article 16j alinéa 2 lettre c, dans lequel nous avons exclu de la qualité pour recourir contre l'approbation des plans, les parties ayant un intérêt juridiquement digne de protection, mais aussi, d'autre part, du nouvel ajout que nous avons validé aujourd'hui à l'alinéa 3, qui limite les griefs invocables aux seuls intérêts individuels dignes de protection. Une restriction du droit de recours est déjà opérée dans la loi sur les installations électriques.
+Je vous prie de ne pas faire un pas supplémentaire et de ne pas "en rajouter une couche" dans la loi sur le Tribunal fédéral en soutenant ma minorité.
 </t>
   </si>
 </sst>
@@ -437,8 +500,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I20" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I24" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I24"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1312,6 +1375,122 @@
         <v>89</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>90</v>
+      </c>
+      <c r="B21" s="1" t="n">
+        <v>46183</v>
+      </c>
+      <c r="C21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" t="s">
+        <v>91</v>
+      </c>
+      <c r="E21" t="s">
+        <v>19</v>
+      </c>
+      <c r="F21" t="s">
+        <v>48</v>
+      </c>
+      <c r="G21" t="s">
+        <v>14</v>
+      </c>
+      <c r="H21" t="s">
+        <v>92</v>
+      </c>
+      <c r="I21" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>94</v>
+      </c>
+      <c r="B22" s="1" t="n">
+        <v>46183</v>
+      </c>
+      <c r="C22" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" t="s">
+        <v>30</v>
+      </c>
+      <c r="E22" t="s">
+        <v>19</v>
+      </c>
+      <c r="F22" t="s">
+        <v>20</v>
+      </c>
+      <c r="G22" t="s">
+        <v>20</v>
+      </c>
+      <c r="H22" t="s">
+        <v>95</v>
+      </c>
+      <c r="I22" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>97</v>
+      </c>
+      <c r="B23" s="1" t="n">
+        <v>46183</v>
+      </c>
+      <c r="C23" t="s">
+        <v>19</v>
+      </c>
+      <c r="D23" t="s">
+        <v>30</v>
+      </c>
+      <c r="E23" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" t="s">
+        <v>20</v>
+      </c>
+      <c r="G23" t="s">
+        <v>20</v>
+      </c>
+      <c r="H23" t="s">
+        <v>98</v>
+      </c>
+      <c r="I23" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>100</v>
+      </c>
+      <c r="B24" s="1" t="n">
+        <v>46183</v>
+      </c>
+      <c r="C24" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" t="s">
+        <v>30</v>
+      </c>
+      <c r="E24" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" t="s">
+        <v>20</v>
+      </c>
+      <c r="G24" t="s">
+        <v>20</v>
+      </c>
+      <c r="H24" t="s">
+        <v>101</v>
+      </c>
+      <c r="I24" t="s">
+        <v>102</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>